<commit_message>
Apply triplet-based content to all 40 category files; rebuild archive
Merge tripl-derived content (hero passport, TL;DR, expert quote, how-to,
FAQ capsules, SEO, type comparison) from 40 content JSONs into the Excel
files; real products and ratings preserved. Add 40 tripl-*.md analyses.
Rebuild medford_categories_all.zip.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012Rw9dvcAKokoAsKsBSt35U
</commit_message>
<xml_diff>
--- a/medford_aspiratory_irrigatory.xlsx
+++ b/medford_aspiratory_irrigatory.xlsx
@@ -941,7 +941,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1022,12 +1022,12 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Как выбрать аспираторы-ирригаторы для клиники?</t>
+          <t>Что делает аспиратор-ирригатор?</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Выбор зависит от задач отделения, совместимости с оборудованием и ключевых характеристик (Страна производства, Производитель, Режим работы). Учитывайте бренд, гарантию, сервис и наличие РУ. Поможем сравнить модели и подобрать оптимальную.</t>
+          <t>Аппарат совмещает ирригацию — подачу стерильного промывочного раствора в операционную зону — и аспирацию — удаление жидкости, крови и мелких частиц тканей за счёт отрицательного давления. Это поддерживает чистоту операционного поля и хорошую видимость при малоинвазивных эндоскопических вмешательствах.</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -1060,12 +1060,12 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Нужно ли регистрационное удостоверение (РУ)?</t>
+          <t>Чем отличаются независимые каналы от общих?</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Да. Это медицинское изделие; для закупки в клинику с медицинской лицензией необходимо действующее регистрационное удостоверение Росздравнадзора. Проверяйте наличие РУ на конкретную модель.</t>
+          <t>В базовых моделях аспирация и ирригация управляются совместно. В продвинутых каналы независимы: давление подачи раствора и разрежение аспирации настраиваются раздельно. Независимость даёт точный контроль поля под конкретный этап операции и тип ткани, что важно в деликатных зонах.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -1098,12 +1098,12 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Какие бренды представлены в каталоге?</t>
+          <t>В каких операциях применяют такие системы?</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>В каталоге представлены модели ведущих производителей. Подберём под ваши задачи и бюджет.</t>
+          <t>Особенно активно — в лапароскопической хирургии, а также в гистероскопии, гастроэнтерологии, урологии, гинекологии и ЛОР-практике. Задача во всех случаях одна: промывать зону, удалять кровь и частицы, проводить лаваж и поддерживать видимость на протяжении процедуры. Профиль вмешательств задаёт требования к модели.</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -1136,12 +1136,12 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Сколько стоит оборудование?</t>
+          <t>Что такое защита от переполнения и сброс вакуума?</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Цена указывается по запросу и зависит от модели, комплектации и условий поставки. Отправьте запрос — подготовим коммерческое предложение за 1 день.</t>
+          <t>Защита от переполнения — сигнализация и автоотключение при заполнении ёмкости, чтобы жидкость не попала в аппарат. Система сброса вакуума безопасно выравнивает давление в канале аспирации до атмосферного. Дополнительно бактериальные фильтры защищают прибор от попадания жидкости и загрязнений.</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -1174,12 +1174,12 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Есть ли гарантия, сервис и обучение?</t>
+          <t>Как управляют аспиратором-ирригатором?</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Да. Обеспечиваем доставку по России, монтаж и ввод в эксплуатацию, обучение персонала, гарантийное и постгарантийное обслуживание, поставку расходных материалов. Телефон: +7 (499) 495-48-21.</t>
+          <t>Управление реализуют с панели прибора, с эндоскопического инструмента или педалью. Управление с инструмента или педали освобождает руки хирурга и ускоряет работу в поле. Часть моделей поддерживает несколько способов; удобный вариант выбирают под привычки операционной бригады.</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -1188,6 +1188,82 @@
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>FAQ_06</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>160</v>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Совместим ли аппарат с моим инструментарием?</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Совместимость зависит от типа канюль, трубок и эндоскопического инструментария. Модели рассчитаны на работу с определёнными расходниками и наборами. Сообщите, какой инструментарий используете, и мы сверим совместимость канюль и трубок до поставки, чтобы расходники не пришлось искать отдельно.</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>aspiratory_irrigatory</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>FAQ_07</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>170</v>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Нужно ли РУ и что с гарантией?</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Аспиратор-ирригатор — медицинское изделие, для применения нужно действующее РУ Росздравнадзора. На поставляемое оборудование распространяется гарантия, а обслуживание и ремонт выполняет собственный инженерный сервис. Реквизиты РУ, срок гарантии и условия по конкретной модели уточняйте у менеджера. Отдельно оговаривают обслуживание насосной части и замену бактериальных фильтров.</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>aspiratory_irrigatory</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>FAQ</t>
         </is>
@@ -2072,7 +2148,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Аспираторы-ирригаторы для оснащения клиник и медицинских учреждений.</t>
+          <t>Аспираторы-ирригаторы эндоскопические — это аппараты, совмещающие подачу промывочного раствора (ирригацию) и удаление жидкости из операционного поля (аспирацию) при малоинвазивных вмешательствах. В каталоге представлены отечественные модели: аспиратор-ирригатор НПФ Крыло АИ-01 «КРЫЛО», аспиратор НПФ Крыло КРАс 1001 и аспиратор-ирригатор ELEPS АИЭ-15/15 с повторно-кратковременным режимом работы (цикл 50 минут работы, 10 минут перерыв). Такие системы поддерживают чистоту поля и видимость в ходе процедуры.</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -2644,7 +2720,7 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Что такое аспираторы-ирригаторы</t>
+          <t>Коротко о категории</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr"/>
@@ -3158,7 +3234,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M24"/>
+  <dimension ref="A1:M25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3484,12 +3560,12 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Тип и назначение</t>
+          <t>Определите тип вмешательств</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Определите задачи, под которые подбирается аспираторы-ирригаторы: профиль отделения, поток и характер исследований или процедур.</t>
+          <t>Требования к прибору зависят от операций: лапароскопия, гистероскопия, урология, гинекология или ЛОР задают нужную производительность и набор функций. Для лапароскопии важен стабильный поток и разрежение. Определите профиль вмешательств до выбора модели — от него зависят каналы и мощность.</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr"/>
@@ -3529,12 +3605,12 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Совместимость с оборудованием</t>
+          <t>Выберите схему каналов</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Проверьте совместимость с имеющейся техникой, платформой и разъёмами — это исключит лишние затраты на дооснащение.</t>
+          <t>Базовые модели совмещают аспирацию и ирригацию с общим управлением, продвинутые дают независимые каналы с раздельной настройкой. Независимость позволяет точно задавать давление подачи и разрежение отдельно под задачу. Если нужен тонкий контроль поля, выбирайте модель с раздельными каналами.</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr"/>
@@ -3574,12 +3650,12 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Ключевые характеристики</t>
+          <t>Оцените регулировку давления и разрежения</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Сравните ключевые параметры моделей: Страна производства, Производитель, Режим работы. Значения — в таблице сравнения и карточках товаров.</t>
+          <t>Плавная настройка разрежения для аспирации и давления для ирригации позволяет подстраивать прибор под этап операции и тип ткани. Уточните диапазоны и способ регулировки (панель, электроника). Точная регулировка важна для деликатных зон и стабильной видимости поля.</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr"/>
@@ -3619,12 +3695,12 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Бренд и качество</t>
+          <t>Проверьте защиту от переполнения и сброс вакуума</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Выбор бренда влияет на ресурс, сервис и совместимость.</t>
+          <t>Защита от переполнения — звуковая или световая сигнализация и автоотключение при заполнении ёмкости — предотвращает попадание жидкости в аппарат. Система сброса вакуума безопасно выравнивает давление в канале аспирации до атмосферного. Уточните наличие этих узлов и бактериальных фильтров.</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr"/>
@@ -3664,12 +3740,12 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Регистрация и допуск</t>
+          <t>Выберите способ управления</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Для клиники с медицинской лицензией необходимо действующее регистрационное удостоверение (РУ) Росздравнадзора на модель.</t>
+          <t>Управление может быть с панели прибора, с эндоскопического инструмента или педалью. Управление с инструмента или педали освобождает руки хирурга и ускоряет работу. Выберите удобный для бригады вариант; часть моделей поддерживает несколько способов одновременно.</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr"/>
@@ -3709,12 +3785,12 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Гарантия и сервис</t>
+          <t>Сверьте совместимость, режим работы и РУ</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Уточняйте гарантию, наличие сервисной поддержки и поставку расходных материалов до закупки.</t>
+          <t>Проверьте совместимость с вашими канюлями, трубками и эндоскопическим инструментарием, чтобы расходники не пришлось искать отдельно. Учтите режим работы: например, ELEPS АИЭ-15/15 рассчитан на повторно-кратковременный цикл 50 минут работы и 10 минут перерыва. Уточните действующее РУ Росздравнадзора до покупки — без него прибор нельзя применять в клинике.</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr"/>
@@ -3764,7 +3840,7 @@
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>Аспираторы-ирригаторы подбирают под задачи отделения и совместимость с имеющимся оборудованием. При выборе обращают внимание на страна производства, производитель, режим работы, а также на наличие регистрационного удостоверения и условия сервиса. Поможем сравнить модели и подобрать оптимальную под ваш поток исследований и бюджет.</t>
+          <t>В аспираторе-ирригаторе я советую смотреть на независимость каналов и способ управления. Раздельная регулировка разрежения и давления позволяет точно настроить прибор под этап операции, а управление с инструмента или педали освобождает руки хирурга. Обязательны защита от переполнения и бактериальные фильтры — это безопасность аппарата и пациента. Совместимость канюль и трубок с вашим инструментарием я проверяю до поставки, иначе расходники придётся искать отдельно.</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
@@ -4048,13 +4124,13 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Что такое аспираторы-ирригаторы</t>
+          <t>Коротко о категории</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr"/>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>Аспираторы-ирригаторы — медицинское оборудование для оснащения клиник и медицинских учреждений. В каталоге Medford представлены модели ведущих производителей. Подберём вариант под задачи вашего отделения.</t>
+          <t>Аспиратор-ирригатор эндоскопический совмещает две функции: ирригацию — подачу стерильного раствора в операционную зону — и аспирацию — удаление жидкости, крови и частиц тканей за счёт разрежения. Аппарат имеет два канала, в продвинутых моделях они управляются независимо. Оборудование поддерживает чистоту поля и видимость при лапароскопии, а также в гинекологии, урологии и ЛОР. При выборе смотрят на независимость каналов, регулировку давления и разрежения, защиту от переполнения и совместимость с инструментарием. Требуется РУ Росздравнадзора.</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
@@ -4091,13 +4167,13 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Как выбрать и на что смотреть</t>
+          <t>Что такое эндоскопический аспиратор-ирригатор</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr"/>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>При выборе оценивают назначение и совместимость с имеющимся оборудованием, ключевые характеристики (Страна производства, Производитель, Режим работы), бренд, наличие РУ, гарантию и сервис.</t>
+          <t>Эндоскопический аспиратор-ирригатор — устройство, совмещающее ирригацию (подачу стерильного промывочного раствора в операционную область) и аспирацию (удаление жидкости и содержимого за счёт отрицательного давления). Оборудование незаменимо при малоинвазивных вмешательствах, когда нужно поддерживать чистоту операционного поля и хорошую визуализацию для хирурга.</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
@@ -4134,13 +4210,13 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Оснащение и совместимость</t>
+          <t>Как это работает</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr"/>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>Уточняйте комплектацию, совместимость с вашей техникой и наличие расходных материалов. Специалисты Medford помогут собрать рабочее решение под ваш профиль.</t>
+          <t>Аппарат имеет два функциональных канала. Канал ирригации создаёт поток раствора, который через трубочную систему и канюлю подаётся в рабочую зону. Канал аспирации формирует разрежение, за счёт которого жидкость выводится через аспирационную канюлю в ёмкость для сбора. В продвинутых моделях процессы контролируются независимо.</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
@@ -4177,13 +4253,13 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>Оплата и доставка</t>
+          <t>Ключевые особенности моделей</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr"/>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>Оплата — по счёту для юридических лиц и ИП. Доставка по всей России, монтаж и ввод в эксплуатацию. Гарантийное и постгарантийное обслуживание, обучение персонала. Телефон для консультаций: +7 (499) 495-48-21.</t>
+          <t>При выборе смотрят на независимость каналов аспирации и ирригации, плавную регулировку разрежения и давления, защиту от переполнения (сигнализация и автоотключение), систему сброса вакуума, способ управления (панель, инструмент, педаль), бактериальные фильтры и совместимость с эндоскопическим инструментарием. Эти узлы определяют точность и безопасность работы.</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
@@ -4200,6 +4276,49 @@
       <c r="K24" s="3" t="inlineStr"/>
       <c r="L24" s="3" t="inlineStr"/>
       <c r="M24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>SEO_05</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>550</v>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Модели каталога и области применения</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr"/>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>В каталоге отечественные решения: аспиратор-ирригатор НПФ Крыло АИ-01 «КРЫЛО», аспиратор НПФ Крыло КРАс 1001 для хирургии и аспиратор-ирригатор ELEPS АИЭ-15/15 с повторно-кратковременным режимом (цикл 50 минут работы, 10 минут перерыв). Системы применяют в лапароскопии, а также в гинекологии, урологии, гастроэнтерологии и ЛОР.</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>aspiratory_irrigatory</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>SEO</t>
+        </is>
+      </c>
+      <c r="J25" s="3" t="inlineStr"/>
+      <c r="K25" s="3" t="inlineStr"/>
+      <c r="L25" s="3" t="inlineStr"/>
+      <c r="M25" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>